<commit_message>
docs: status talking agent + laporan Ngobrol dengan AI (3 Sep 2026); env GROQ di infra README
CLAUDE.md: [x] Fallback reconcile + [x] Laporan Ngobrol dengan AI (3 permukaan,
GRADED-only, tanpa ranking) + backlog disesuaikan (list transcript-level tetap
luar scope). infra/README: baris GROQ_API_KEY (speaking). Template soal refresh.

Co-Authored-By: Claude Code <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/deliverables/template-soal-v1.xlsx
+++ b/deliverables/template-soal-v1.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="96">
   <si>
     <t>lesson_code</t>
   </si>
@@ -227,6 +227,33 @@
     <t>MEMO: The monthly meeting is moved. It will be held on Wednesday at 10 AM in Room 3.</t>
   </si>
   <si>
+    <t>SPK-01</t>
+  </si>
+  <si>
+    <t>Berlatih Bicara</t>
+  </si>
+  <si>
+    <t>Speaking English</t>
+  </si>
+  <si>
+    <t>A1</t>
+  </si>
+  <si>
+    <t>speaking</t>
+  </si>
+  <si>
+    <t>ucapan</t>
+  </si>
+  <si>
+    <t>Baca kalimat ini dengan lantang.</t>
+  </si>
+  <si>
+    <t>I will call you tomorrow</t>
+  </si>
+  <si>
+    <t>Latihan pelafalan: ucapkan dengan jelas, jangan terburu-buru.</t>
+  </si>
+  <si>
     <t>Kolom</t>
   </si>
   <si>
@@ -254,7 +281,7 @@
     <t>Hanya untuk pilihan_ganda. Keempatnya wajib diisi.</t>
   </si>
   <si>
-    <t>pilihan_ganda: A/B/C/D · isian: jawaban utama · susun_kalimat: kalimat lengkap yang benar (min. 3 kata).</t>
+    <t>pilihan_ganda: A/B/C/D · isian: jawaban utama · susun_kalimat: kalimat lengkap (min. 3 kata) · ucapan: kalimat yang harus diucapkan karyawan (min. 2 kata).</t>
   </si>
   <si>
     <t>Hanya isian: variasi jawaban yang diterima, dipisah titik-koma. Contoh: submit;send</t>
@@ -267,6 +294,12 @@
   </si>
   <si>
     <t>Teks bacaan untuk soal reading. Kosongkan jika tidak ada.</t>
+  </si>
+  <si>
+    <t>Prompt = instruksi (mis. "Baca kalimat ini dengan lantang."). Answer = kalimat yang diucapkan. Audio contoh opsional via media_file (mp3/m4a).</t>
+  </si>
+  <si>
+    <t>Tambahan: speaking (soal ucapan).</t>
   </si>
 </sst>
 </file>
@@ -647,7 +680,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:R500"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="12" customWidth="1"/>
@@ -1003,500 +1036,62 @@
         <v>70</v>
       </c>
     </row>
-    <row r="7" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="8" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="9" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="10" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="11" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="12" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="13" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="17" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="18" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="22" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="23" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="24" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="25" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="26" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="27" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="33" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="34" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="35" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="36" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="37" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="38" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="39" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="40" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="41" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="43" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="44" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="45" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="46" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="47" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="48" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="49" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="50" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="51" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="52" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="53" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="54" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="55" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="56" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="57" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="58" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="59" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="60" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="61" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="62" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="63" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="64" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="65" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="66" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="67" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="68" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="69" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="70" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="71" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="72" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="73" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="74" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="75" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="76" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="77" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="78" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="79" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="80" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="81" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="82" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="83" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="84" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="85" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="86" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="87" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="88" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="89" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="90" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="91" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="92" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="93" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="94" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="95" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="96" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="97" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="98" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="99" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="100" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="101" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="102" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="103" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="104" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="105" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="106" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="107" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="108" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="109" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="110" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="111" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="112" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="113" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="114" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="115" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="116" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="117" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="118" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="119" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="120" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="121" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="122" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="123" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="124" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="125" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="126" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="127" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="128" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="129" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="130" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="131" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="132" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="133" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="134" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="135" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="136" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="137" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="138" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="139" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="140" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="141" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="145" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="146" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="147" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="148" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="149" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="150" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="151" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="152" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="153" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="154" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="155" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="156" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="157" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="158" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="159" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="160" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="161" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="162" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="163" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="164" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="165" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="166" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="167" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="168" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="169" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="170" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="171" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="172" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="173" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="174" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="175" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="176" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="177" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="178" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="179" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="180" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="181" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="182" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="183" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="184" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="185" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="186" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="187" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="188" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="189" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="190" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="191" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="192" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="193" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="194" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="195" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="196" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="197" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="198" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="199" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="200" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="201" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="202" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="203" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="209" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="210" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="211" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="212" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="213" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="214" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="215" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="216" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="217" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="218" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="219" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="220" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="221" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="222" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="223" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="224" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="225" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="226" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="227" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="228" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="229" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="230" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="231" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="232" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="233" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="234" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="235" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="236" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="237" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="238" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="239" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="240" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="241" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="242" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="243" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="244" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="245" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="246" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="247" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="248" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="249" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="250" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="251" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="252" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="253" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="254" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="255" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="256" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="257" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="258" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="259" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="260" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="261" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="262" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="263" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="264" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="265" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="266" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="267" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="268" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="269" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="270" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="271" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="272" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="273" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="274" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="275" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="276" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="277" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="278" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="279" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="280" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="281" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="282" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="283" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="284" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="285" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="286" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="287" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="288" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="289" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="290" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="291" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="292" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="293" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="294" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="295" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="296" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="297" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="298" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="299" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="300" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="301" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="302" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="303" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="304" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="305" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="306" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="307" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="308" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="309" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="310" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="311" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="312" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="313" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="314" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="315" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="316" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="317" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="318" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="319" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="320" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="321" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="322" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="323" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="324" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="325" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="326" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="327" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="328" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="329" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="330" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="331" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="332" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="333" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="334" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="335" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="336" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="337" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="338" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="339" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="340" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="341" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="342" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="343" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="344" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="345" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="346" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="347" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="348" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="349" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="350" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="351" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="352" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="353" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="354" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="355" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="356" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="357" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="358" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="359" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="360" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="361" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="362" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="363" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="364" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="365" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="366" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="367" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="368" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="369" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="370" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="371" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="372" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="373" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="374" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="375" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="376" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="377" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="378" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="379" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="380" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="381" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="382" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="383" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="384" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="385" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="386" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="387" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="388" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="389" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="390" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="391" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="392" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="393" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="394" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="395" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="396" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="397" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="398" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="399" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="400" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="401" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="402" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="403" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="404" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="405" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="406" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="407" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="408" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="409" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="410" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="411" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="412" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="413" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="414" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="415" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="416" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="417" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="418" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="419" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="420" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="421" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="422" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="423" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="424" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="425" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="426" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="427" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="428" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="429" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="430" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="431" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="432" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="433" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="434" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="435" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="436" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="437" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="438" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="439" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="440" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="441" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="442" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="443" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="444" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="445" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="446" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="447" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="448" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="449" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="450" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="451" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="452" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="453" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="454" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="455" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="456" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="457" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="458" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="459" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="460" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="461" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="462" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="463" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="464" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="465" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="466" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="467" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="468" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="469" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="470" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="471" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="472" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="473" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="474" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="475" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="476" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="477" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="478" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="479" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="480" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="481" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="482" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="483" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="484" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="485" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="486" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="487" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="488" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="489" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="490" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="491" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="492" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="493" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="494" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="495" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="496" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="497" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="498" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="499" spans="4:8" x14ac:dyDescent="0.25"/>
-    <row r="500" spans="4:8" x14ac:dyDescent="0.25"/>
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>71</v>
+      </c>
+      <c r="B7" t="s">
+        <v>72</v>
+      </c>
+      <c r="C7" t="s">
+        <v>73</v>
+      </c>
+      <c r="D7" t="s">
+        <v>48</v>
+      </c>
+      <c r="E7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" t="s">
+        <v>24</v>
+      </c>
+      <c r="H7" t="s">
+        <v>76</v>
+      </c>
+      <c r="I7" t="s">
+        <v>77</v>
+      </c>
+      <c r="J7" t="s">
+        <v>32</v>
+      </c>
+      <c r="K7" t="s">
+        <v>32</v>
+      </c>
+      <c r="L7" t="s">
+        <v>32</v>
+      </c>
+      <c r="M7" t="s">
+        <v>32</v>
+      </c>
+      <c r="N7" t="s">
+        <v>78</v>
+      </c>
+      <c r="O7" t="s">
+        <v>32</v>
+      </c>
+      <c r="P7" t="s">
+        <v>79</v>
+      </c>
+      <c r="Q7" t="s">
+        <v>32</v>
+      </c>
+      <c r="R7" t="s">
+        <v>32</v>
+      </c>
+    </row>
   </sheetData>
   <dataValidations count="8">
     <dataValidation type="list" allowBlank="1" sqref="D10:D500">
@@ -1512,26 +1107,26 @@
       <formula1>"A1,A2,B1,B2,C1,C2"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="F10:F500">
-      <formula1>"vocabulary,grammar,listening,reading"</formula1>
+      <formula1>"vocabulary,grammar,listening,reading,speaking"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="F2:F500">
-      <formula1>"vocabulary,grammar,listening,reading"</formula1>
+      <formula1>"vocabulary,grammar,listening,reading,speaking"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H10:H500">
-      <formula1>"pilihan_ganda,isian,susun_kalimat"</formula1>
+      <formula1>"pilihan_ganda,isian,susun_kalimat,ucapan"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="H2:H500">
-      <formula1>"pilihan_ganda,isian,susun_kalimat"</formula1>
+      <formula1>"pilihan_ganda,isian,susun_kalimat,ucapan"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B11"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="22" customWidth="1"/>
@@ -1540,10 +1135,10 @@
   <sheetData>
     <row r="1" spans="1:2" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>71</v>
+        <v>80</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>72</v>
+        <v>81</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -1551,15 +1146,15 @@
         <v>0</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>82</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>74</v>
+        <v>83</v>
       </c>
       <c r="B3" t="s">
-        <v>75</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.25">
@@ -1567,7 +1162,7 @@
         <v>6</v>
       </c>
       <c r="B4" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.25">
@@ -1575,15 +1170,15 @@
         <v>8</v>
       </c>
       <c r="B5" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="B6" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.25">
@@ -1591,7 +1186,7 @@
         <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>80</v>
+        <v>89</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -1599,7 +1194,7 @@
         <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
@@ -1607,7 +1202,7 @@
         <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>82</v>
+        <v>91</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
@@ -1615,7 +1210,7 @@
         <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>83</v>
+        <v>92</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -1623,11 +1218,27 @@
         <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>84</v>
+        <v>93</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>76</v>
+      </c>
+      <c r="B12" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>5</v>
+      </c>
+      <c r="B13" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>